<commit_message>
added languauge / topic selector.
</commit_message>
<xml_diff>
--- a/excel/armenian_history_timeline.xlsx
+++ b/excel/armenian_history_timeline.xlsx
@@ -8,12 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Armenian_History\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81821040-2A7E-4348-BD40-56B20804A142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F79F36BF-9BEC-4606-8D7F-96624D8F5B67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CB6D9F54-74F6-4429-8058-546C957028B6}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="619" xr2:uid="{CB6D9F54-74F6-4429-8058-546C957028B6}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="hist" sheetId="1" r:id="rId1"/>
+    <sheet name="hist_translation" sheetId="2" r:id="rId2"/>
+    <sheet name="leaders" sheetId="3" r:id="rId3"/>
+    <sheet name="flag" sheetId="5" r:id="rId4"/>
+    <sheet name="map" sheetId="7" r:id="rId5"/>
+    <sheet name="population" sheetId="17" r:id="rId6"/>
+    <sheet name="gdp" sheetId="18" r:id="rId7"/>
+    <sheet name="stem" sheetId="9" r:id="rId8"/>
+    <sheet name="sports" sheetId="11" r:id="rId9"/>
+    <sheet name="music" sheetId="13" r:id="rId10"/>
+    <sheet name="literature" sheetId="15" r:id="rId11"/>
+    <sheet name="people_translation_desc" sheetId="4" r:id="rId12"/>
+    <sheet name="flag_translation_desc" sheetId="6" r:id="rId13"/>
+    <sheet name="map_translation_desc" sheetId="8" r:id="rId14"/>
+    <sheet name="stem_translation_desc" sheetId="10" r:id="rId15"/>
+    <sheet name="sports_translation_desc" sheetId="12" r:id="rId16"/>
+    <sheet name="music_translation_desc" sheetId="14" r:id="rId17"/>
+    <sheet name="literature_translation_desc" sheetId="16" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,70 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="44">
-  <si>
-    <t>timeline_start</t>
-  </si>
-  <si>
-    <t>timeline_finish</t>
-  </si>
-  <si>
-    <t>timeline_description</t>
-  </si>
-  <si>
-    <t>timeline_0001</t>
-  </si>
-  <si>
-    <t>timeline_id</t>
-  </si>
-  <si>
-    <t>timeline_0002</t>
-  </si>
-  <si>
-    <t>timeline_0003</t>
-  </si>
-  <si>
-    <t>timeline_0004</t>
-  </si>
-  <si>
-    <t>timeline_0005</t>
-  </si>
-  <si>
-    <t>timeline_0006</t>
-  </si>
-  <si>
-    <t>timeline_0007</t>
-  </si>
-  <si>
-    <t>timeline_0008</t>
-  </si>
-  <si>
-    <t>timeline_0009</t>
-  </si>
-  <si>
-    <t>timeline_0010</t>
-  </si>
-  <si>
-    <t>timeline_0011</t>
-  </si>
-  <si>
-    <t>timeline_0012</t>
-  </si>
-  <si>
-    <t>timeline_0013</t>
-  </si>
-  <si>
-    <t>timeline_0014</t>
-  </si>
-  <si>
-    <t>timeline_0015</t>
-  </si>
-  <si>
-    <t>timeline_0016</t>
-  </si>
-  <si>
-    <t>timeline_0017</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="60">
   <si>
     <t>Մ՛իջին հին քարի դա րի' պալեոլիթի մ ո լս ֊ 
 տ իերյա ն մշա կույթի գոյա տ ևմա ն ժա մա նա կա շրջա ն։</t>
@@ -138,19 +92,7 @@
 ցեղերի հա նդես գալը Փոքր Ա սիա յում։</t>
   </si>
   <si>
-    <t>ՄԵՐ ԹՎԱԿԱՆՈԻԹ8ՈԻՆԻ8 ԱՌԱՏ</t>
-  </si>
-  <si>
-    <t>timeline_section_title</t>
-  </si>
-  <si>
-    <t>timeline_section_id</t>
-  </si>
-  <si>
     <t>BCE</t>
-  </si>
-  <si>
-    <t>ՄԵՐ ԹվԱԿԱնՈԻԹՅՈԻՆ</t>
   </si>
   <si>
     <t>CE</t>
@@ -178,6 +120,131 @@
   <si>
     <t>Հ ա յա ս ա ֊Ա ղ ղ ի ց ե ղ ա յի . 
 . միութ յա ն գո յո ւթ յա ն ժա մա նա կա շրջա նը։</t>
+  </si>
+  <si>
+    <t>history_0001</t>
+  </si>
+  <si>
+    <t>history_0002</t>
+  </si>
+  <si>
+    <t>history_0003</t>
+  </si>
+  <si>
+    <t>history_0004</t>
+  </si>
+  <si>
+    <t>history_0005</t>
+  </si>
+  <si>
+    <t>history_0006</t>
+  </si>
+  <si>
+    <t>history_0007</t>
+  </si>
+  <si>
+    <t>history_0008</t>
+  </si>
+  <si>
+    <t>history_0009</t>
+  </si>
+  <si>
+    <t>history_0010</t>
+  </si>
+  <si>
+    <t>history_0011</t>
+  </si>
+  <si>
+    <t>history_0012</t>
+  </si>
+  <si>
+    <t>history_0013</t>
+  </si>
+  <si>
+    <t>history_0014</t>
+  </si>
+  <si>
+    <t>history_0015</t>
+  </si>
+  <si>
+    <t>history_0016</t>
+  </si>
+  <si>
+    <t>history_0017</t>
+  </si>
+  <si>
+    <t>history_id</t>
+  </si>
+  <si>
+    <t>history_section_title</t>
+  </si>
+  <si>
+    <t>history_section_id</t>
+  </si>
+  <si>
+    <t>history_description</t>
+  </si>
+  <si>
+    <t>history_start</t>
+  </si>
+  <si>
+    <t>history_finish</t>
+  </si>
+  <si>
+    <t>leaders_id</t>
+  </si>
+  <si>
+    <t>leaders_section_title</t>
+  </si>
+  <si>
+    <t>leaders_section_id</t>
+  </si>
+  <si>
+    <t>leaders_start</t>
+  </si>
+  <si>
+    <t>leaders_finish</t>
+  </si>
+  <si>
+    <t>leaders_description</t>
+  </si>
+  <si>
+    <t>leaders_0001</t>
+  </si>
+  <si>
+    <t>history_description_en</t>
+  </si>
+  <si>
+    <t>history_description_ru</t>
+  </si>
+  <si>
+    <t>history_description_ir</t>
+  </si>
+  <si>
+    <t>history_description_fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> է՚գե յա ն ա շխ ա րհից ՛և Բա լկա ններից դեպի 
+Փոքր Ասիսւ շա րժվող ցեղերի նոր ա լիք («Ծ ո վ ի ժողովուրդներ» ) ։</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Մ ուրսիլիս Բ խեթակա՛ն թա գա վորի պ ա տ երա զմները Հա ­
+լա սա ֊Ա զ գ ի ի դ ե մ ւ</t>
+  </si>
+  <si>
+    <t>history_section_en</t>
+  </si>
+  <si>
+    <t>history_section_ru</t>
+  </si>
+  <si>
+    <t>history_section_ir</t>
+  </si>
+  <si>
+    <t>history_section_fr</t>
+  </si>
+  <si>
+    <t>ՄԵՐ ԹՎԱԿԱՆՈԻԹՅՈԻՆԻՑ ԱՌԱՋ</t>
   </si>
 </sst>
 </file>
@@ -219,9 +286,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -556,390 +622,979 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EB90175-CD20-47DA-AE7C-CB0ADADA1BDA}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" customWidth="1"/>
     <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" t="s">
-        <v>1</v>
+        <v>36</v>
+      </c>
+      <c r="B1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" t="s">
+        <v>37</v>
       </c>
       <c r="F1" t="s">
-        <v>2</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" t="s">
-        <v>35</v>
+        <v>11</v>
+      </c>
+      <c r="C2">
+        <v>1000000</v>
       </c>
       <c r="D2">
-        <v>1000000</v>
-      </c>
-      <c r="E2">
         <v>800000</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>23</v>
+      <c r="E2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" t="s">
-        <v>35</v>
+        <v>11</v>
+      </c>
+      <c r="C3">
+        <f>D2</f>
+        <v>800000</v>
       </c>
       <c r="D3">
-        <f>E2</f>
-        <v>800000</v>
-      </c>
-      <c r="E3">
         <v>100000</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>24</v>
+      <c r="E3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" t="s">
-        <v>35</v>
+        <v>11</v>
+      </c>
+      <c r="C4">
+        <f t="shared" ref="C4:C20" si="0">D3</f>
+        <v>100000</v>
       </c>
       <c r="D4">
-        <f t="shared" ref="D4:D18" si="0">E3</f>
-        <v>100000</v>
-      </c>
-      <c r="E4">
         <v>40000</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>21</v>
+      <c r="E4" t="s">
+        <v>59</v>
+      </c>
+      <c r="F4" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" t="s">
-        <v>35</v>
+        <v>11</v>
+      </c>
+      <c r="C5">
+        <v>65000</v>
       </c>
       <c r="D5">
-        <v>65000</v>
-      </c>
-      <c r="E5">
         <v>40000</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>22</v>
+      <c r="E5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" t="s">
-        <v>35</v>
+        <v>11</v>
+      </c>
+      <c r="C6">
+        <f>D4</f>
+        <v>40000</v>
       </c>
       <c r="D6">
-        <f>E4</f>
-        <v>40000</v>
-      </c>
-      <c r="E6">
         <v>12000</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>25</v>
+      <c r="E6" t="s">
+        <v>59</v>
+      </c>
+      <c r="F6" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7">
+        <v>11</v>
+      </c>
+      <c r="C7">
         <f t="shared" si="0"/>
         <v>12000</v>
       </c>
-      <c r="E7">
+      <c r="D7">
         <v>8000</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>26</v>
+      <c r="E7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F7" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C8" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8">
+        <v>11</v>
+      </c>
+      <c r="C8">
         <f t="shared" si="0"/>
         <v>8000</v>
       </c>
-      <c r="E8">
+      <c r="D8">
         <v>5000</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>27</v>
+      <c r="E8" t="s">
+        <v>59</v>
+      </c>
+      <c r="F8" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" t="s">
         <v>11</v>
       </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9">
+      <c r="C9">
         <f t="shared" si="0"/>
         <v>5000</v>
       </c>
-      <c r="E9">
+      <c r="D9">
         <v>5000</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>28</v>
+      <c r="E9" t="s">
+        <v>59</v>
+      </c>
+      <c r="F9" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" t="s">
-        <v>35</v>
+        <v>11</v>
+      </c>
+      <c r="C10">
+        <v>3000</v>
       </c>
       <c r="D10">
         <v>3000</v>
       </c>
-      <c r="E10">
-        <v>3000</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>29</v>
+      <c r="E10" t="s">
+        <v>59</v>
+      </c>
+      <c r="F10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" t="s">
-        <v>35</v>
-      </c>
-      <c r="D11">
+        <v>11</v>
+      </c>
+      <c r="C11">
         <f t="shared" si="0"/>
         <v>3000</v>
       </c>
-      <c r="E11">
+      <c r="D11">
         <v>3000</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>30</v>
+      <c r="E11" t="s">
+        <v>59</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" t="s">
-        <v>35</v>
-      </c>
-      <c r="D12">
+        <v>11</v>
+      </c>
+      <c r="C12">
         <f t="shared" si="0"/>
         <v>3000</v>
       </c>
-      <c r="E12">
+      <c r="D12">
         <v>3000</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>31</v>
+      <c r="E12" t="s">
+        <v>59</v>
+      </c>
+      <c r="F12" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" t="s">
-        <v>35</v>
+        <v>11</v>
+      </c>
+      <c r="C13">
+        <v>2000</v>
       </c>
       <c r="D13">
         <v>2000</v>
       </c>
-      <c r="E13">
-        <v>2000</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>41</v>
+      <c r="E13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F13" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14">
+        <v>11</v>
+      </c>
+      <c r="C14">
         <f t="shared" si="0"/>
         <v>2000</v>
       </c>
-      <c r="E14">
+      <c r="D14">
         <v>2000</v>
       </c>
-      <c r="F14" s="1" t="s">
-        <v>42</v>
+      <c r="E14" t="s">
+        <v>59</v>
+      </c>
+      <c r="F14" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
-      </c>
-      <c r="C15" t="s">
-        <v>35</v>
+        <v>11</v>
+      </c>
+      <c r="C15">
+        <f>D14</f>
+        <v>2000</v>
       </c>
       <c r="D15">
-        <f>E14</f>
-        <v>2000</v>
-      </c>
-      <c r="E15">
         <v>1200</v>
       </c>
-      <c r="F15" s="1" t="s">
-        <v>43</v>
+      <c r="E15" t="s">
+        <v>59</v>
+      </c>
+      <c r="F15" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" t="s">
-        <v>36</v>
-      </c>
-      <c r="C16" t="s">
-        <v>37</v>
+        <v>33</v>
+      </c>
+      <c r="C16">
+        <f t="shared" si="0"/>
+        <v>1200</v>
       </c>
       <c r="D16">
-        <v>1</v>
-      </c>
-      <c r="E16">
-        <v>1</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>38</v>
+        <v>2000</v>
+      </c>
+      <c r="E16" t="s">
+        <v>59</v>
+      </c>
+      <c r="F16" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" t="s">
-        <v>36</v>
-      </c>
-      <c r="C17" t="s">
-        <v>37</v>
+        <v>33</v>
+      </c>
+      <c r="C17">
+        <v>1334</v>
       </c>
       <c r="D17">
-        <v>2</v>
-      </c>
-      <c r="E17">
-        <v>4</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>39</v>
+        <v>1330</v>
+      </c>
+      <c r="E17" t="s">
+        <v>59</v>
+      </c>
+      <c r="F17" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="B18" t="s">
-        <v>36</v>
-      </c>
-      <c r="C18" t="s">
-        <v>37</v>
+        <v>12</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
       </c>
       <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18" t="s">
+        <v>59</v>
+      </c>
+      <c r="F18" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>34</v>
+      </c>
+      <c r="B19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19">
+        <v>2</v>
+      </c>
+      <c r="D19">
+        <v>4</v>
+      </c>
+      <c r="E19" t="s">
+        <v>59</v>
+      </c>
+      <c r="F19" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="E18">
+      <c r="D20">
         <v>6</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>40</v>
+      <c r="E20" t="s">
+        <v>59</v>
+      </c>
+      <c r="F20" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{403EC2D6-EC80-4DF3-A5FC-E8B157AEE389}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15E02974-8D1D-4298-958D-60C87455965E}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AFD9CFB-FFC6-4F39-B470-84B994673B18}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A327C2BD-5A5E-44EA-AA1C-F2C0BF56DFF6}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{687B57B2-1B3E-48BA-824F-AEE04B6BD056}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45180A91-9863-40B5-938E-B206FEF445A3}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1318E309-6B04-4BEA-89E2-6605D2F238B5}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60F89C32-04BC-4837-8FDC-E136A2788C6E}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{905144BE-5622-4537-A3B2-F9445A2BC655}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47C770DC-C83D-496B-828F-72873AF4491D}">
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.140625" customWidth="1"/>
+    <col min="7" max="7" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.5703125" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H1" t="s">
+        <v>58</v>
+      </c>
+      <c r="I1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4DD3433-19D9-48A1-ABD3-10A1A337A3A1}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95F1D444-82B4-47AB-B8A5-89EA287F92A2}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39A92E0F-1F1D-4C14-B6A7-00F32784E78A}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFE901FA-8564-44A3-9100-D50CB00E5FC1}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{531700B1-68CC-4E7F-BDF1-5B34261C6473}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5855070E-1B2E-44AD-B7D0-C252A4C52167}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64982EF2-6B02-49A5-92EA-C16ACA5121CF}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>